<commit_message>
Add GitHub Pages deployment
</commit_message>
<xml_diff>
--- a/static/TALENKAART_DATA/talenkaart_data.xlsx
+++ b/static/TALENKAART_DATA/talenkaart_data.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1243">
   <si>
     <t>Locatie</t>
   </si>
@@ -536,7 +536,7 @@
     <t>fra,spa,dui</t>
   </si>
   <si>
-    <t>nld,tw,eng</t>
+    <t>nld,twi,eng</t>
   </si>
   <si>
     <t>twi,eng</t>
@@ -2232,9 +2232,6 @@
   </si>
   <si>
     <t>Spinoza Lyceum</t>
-  </si>
-  <si>
-    <t>nld,twi,eng</t>
   </si>
   <si>
     <t>nld,pol,eng</t>
@@ -18734,7 +18731,7 @@
       </c>
       <c r="C938" s="3"/>
       <c r="D938" t="s" s="3">
-        <v>731</v>
+        <v>165</v>
       </c>
       <c r="E938" s="4"/>
       <c r="F938" s="4"/>
@@ -18748,7 +18745,7 @@
       </c>
       <c r="C939" s="3"/>
       <c r="D939" t="s" s="3">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E939" s="4"/>
       <c r="F939" s="4"/>
@@ -18860,7 +18857,7 @@
       </c>
       <c r="C947" s="3"/>
       <c r="D947" t="s" s="3">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E947" s="4"/>
       <c r="F947" s="4"/>
@@ -18874,7 +18871,7 @@
       </c>
       <c r="C948" s="3"/>
       <c r="D948" t="s" s="3">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E948" s="4"/>
       <c r="F948" s="4"/>
@@ -18895,7 +18892,7 @@
     </row>
     <row r="950" ht="13.65" customHeight="1">
       <c r="A950" t="s" s="3">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B950" t="s" s="3">
         <v>178</v>
@@ -18909,21 +18906,21 @@
     </row>
     <row r="951" ht="13.65" customHeight="1">
       <c r="A951" t="s" s="3">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B951" t="s" s="3">
         <v>178</v>
       </c>
       <c r="C951" s="3"/>
       <c r="D951" t="s" s="3">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="E951" s="4"/>
       <c r="F951" s="4"/>
     </row>
     <row r="952" ht="13.65" customHeight="1">
       <c r="A952" t="s" s="3">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B952" t="s" s="3">
         <v>178</v>
@@ -18937,7 +18934,7 @@
     </row>
     <row r="953" ht="13.65" customHeight="1">
       <c r="A953" t="s" s="3">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B953" t="s" s="3">
         <v>178</v>
@@ -18951,7 +18948,7 @@
     </row>
     <row r="954" ht="13.65" customHeight="1">
       <c r="A954" t="s" s="3">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B954" t="s" s="3">
         <v>444</v>
@@ -18965,10 +18962,10 @@
     </row>
     <row r="955" ht="13.65" customHeight="1">
       <c r="A955" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B955" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B955" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C955" s="3"/>
       <c r="D955" t="s" s="3">
@@ -18979,10 +18976,10 @@
     </row>
     <row r="956" ht="13.65" customHeight="1">
       <c r="A956" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B956" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B956" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C956" s="3"/>
       <c r="D956" t="s" s="3">
@@ -18993,10 +18990,10 @@
     </row>
     <row r="957" ht="13.65" customHeight="1">
       <c r="A957" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B957" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B957" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C957" s="3"/>
       <c r="D957" t="s" s="3">
@@ -19007,38 +19004,38 @@
     </row>
     <row r="958" ht="13.65" customHeight="1">
       <c r="A958" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B958" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B958" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C958" s="3"/>
       <c r="D958" t="s" s="3">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="E958" s="4"/>
       <c r="F958" s="4"/>
     </row>
     <row r="959" ht="13.65" customHeight="1">
       <c r="A959" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B959" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B959" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C959" s="3"/>
       <c r="D959" t="s" s="3">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="E959" s="4"/>
       <c r="F959" s="4"/>
     </row>
     <row r="960" ht="13.65" customHeight="1">
       <c r="A960" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B960" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B960" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C960" s="3"/>
       <c r="D960" t="s" s="3">
@@ -19049,38 +19046,38 @@
     </row>
     <row r="961" ht="13.65" customHeight="1">
       <c r="A961" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B961" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B961" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C961" s="3"/>
       <c r="D961" t="s" s="3">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="E961" s="4"/>
       <c r="F961" s="4"/>
     </row>
     <row r="962" ht="13.65" customHeight="1">
       <c r="A962" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B962" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B962" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C962" s="3"/>
       <c r="D962" t="s" s="3">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="E962" s="4"/>
       <c r="F962" s="4"/>
     </row>
     <row r="963" ht="13.65" customHeight="1">
       <c r="A963" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B963" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B963" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C963" s="3"/>
       <c r="D963" t="s" s="3">
@@ -19091,10 +19088,10 @@
     </row>
     <row r="964" ht="13.65" customHeight="1">
       <c r="A964" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B964" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B964" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C964" s="3"/>
       <c r="D964" t="s" s="3">
@@ -19105,24 +19102,24 @@
     </row>
     <row r="965" ht="13.65" customHeight="1">
       <c r="A965" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B965" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B965" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C965" s="3"/>
       <c r="D965" t="s" s="3">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="E965" s="4"/>
       <c r="F965" s="4"/>
     </row>
     <row r="966" ht="13.65" customHeight="1">
       <c r="A966" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B966" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B966" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C966" s="3"/>
       <c r="D966" t="s" s="3">
@@ -19133,21 +19130,21 @@
     </row>
     <row r="967" ht="13.65" customHeight="1">
       <c r="A967" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B967" t="s" s="3">
         <v>738</v>
-      </c>
-      <c r="B967" t="s" s="3">
-        <v>739</v>
       </c>
       <c r="C967" s="3"/>
       <c r="D967" t="s" s="3">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E967" s="4"/>
       <c r="F967" s="4"/>
     </row>
     <row r="968" ht="13.65" customHeight="1">
       <c r="A968" t="s" s="3">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B968" t="s" s="3">
         <v>7</v>
@@ -19161,21 +19158,21 @@
     </row>
     <row r="969" ht="13.65" customHeight="1">
       <c r="A969" t="s" s="3">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B969" t="s" s="3">
         <v>444</v>
       </c>
       <c r="C969" s="3"/>
       <c r="D969" t="s" s="3">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="E969" s="4"/>
       <c r="F969" s="4"/>
     </row>
     <row r="970" ht="13.65" customHeight="1">
       <c r="A970" t="s" s="3">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B970" t="s" s="3">
         <v>444</v>
@@ -19189,35 +19186,35 @@
     </row>
     <row r="971" ht="13.65" customHeight="1">
       <c r="A971" t="s" s="3">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B971" t="s" s="3">
         <v>444</v>
       </c>
       <c r="C971" s="3"/>
       <c r="D971" t="s" s="3">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="E971" s="4"/>
       <c r="F971" s="4"/>
     </row>
     <row r="972" ht="13.65" customHeight="1">
       <c r="A972" t="s" s="3">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B972" t="s" s="3">
         <v>444</v>
       </c>
       <c r="C972" s="3"/>
       <c r="D972" t="s" s="3">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="E972" s="4"/>
       <c r="F972" s="4"/>
     </row>
     <row r="973" ht="13.65" customHeight="1">
       <c r="A973" t="s" s="3">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B973" t="s" s="3">
         <v>444</v>
@@ -19231,35 +19228,35 @@
     </row>
     <row r="974" ht="13.65" customHeight="1">
       <c r="A974" t="s" s="3">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B974" t="s" s="3">
         <v>444</v>
       </c>
       <c r="C974" s="3"/>
       <c r="D974" t="s" s="3">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="E974" s="4"/>
       <c r="F974" s="4"/>
     </row>
     <row r="975" ht="13.65" customHeight="1">
       <c r="A975" t="s" s="3">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B975" t="s" s="3">
         <v>444</v>
       </c>
       <c r="C975" s="3"/>
       <c r="D975" t="s" s="3">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="E975" s="4"/>
       <c r="F975" s="4"/>
     </row>
     <row r="976" ht="13.65" customHeight="1">
       <c r="A976" t="s" s="3">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B976" t="s" s="3">
         <v>444</v>
@@ -19273,7 +19270,7 @@
     </row>
     <row r="977" ht="13.65" customHeight="1">
       <c r="A977" t="s" s="3">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B977" t="s" s="3">
         <v>178</v>
@@ -19287,21 +19284,21 @@
     </row>
     <row r="978" ht="13.65" customHeight="1">
       <c r="A978" t="s" s="3">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B978" t="s" s="3">
         <v>178</v>
       </c>
       <c r="C978" s="3"/>
       <c r="D978" t="s" s="3">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="E978" s="4"/>
       <c r="F978" s="4"/>
     </row>
     <row r="979" ht="13.65" customHeight="1">
       <c r="A979" t="s" s="3">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B979" t="s" s="3">
         <v>178</v>
@@ -19315,14 +19312,14 @@
     </row>
     <row r="980" ht="13.65" customHeight="1">
       <c r="A980" t="s" s="3">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B980" t="s" s="3">
         <v>178</v>
       </c>
       <c r="C980" s="3"/>
       <c r="D980" t="s" s="3">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="E980" s="4"/>
       <c r="F980" s="4"/>
@@ -19336,7 +19333,7 @@
       </c>
       <c r="C981" s="3"/>
       <c r="D981" t="s" s="3">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="E981" s="4"/>
       <c r="F981" s="4"/>
@@ -19366,16 +19363,16 @@
   <sheetData>
     <row r="1" ht="13.65" customHeight="1">
       <c r="A1" t="s" s="2">
+        <v>758</v>
+      </c>
+      <c r="B1" t="s" s="2">
         <v>759</v>
-      </c>
-      <c r="B1" t="s" s="2">
-        <v>760</v>
       </c>
       <c r="C1" t="s" s="2">
         <v>1</v>
       </c>
       <c r="D1" t="s" s="2">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="E1" s="4"/>
     </row>
@@ -19384,13 +19381,13 @@
         <v>6</v>
       </c>
       <c r="B2" t="s" s="3">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="C2" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D2" t="s" s="3">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="E2" s="4"/>
     </row>
@@ -19399,43 +19396,43 @@
         <v>177</v>
       </c>
       <c r="B3" t="s" s="3">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="C3" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D3" t="s" s="3">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="E3" s="4"/>
     </row>
     <row r="4" ht="13.65" customHeight="1">
       <c r="A4" t="s" s="3">
+        <v>764</v>
+      </c>
+      <c r="B4" t="s" s="6">
         <v>765</v>
-      </c>
-      <c r="B4" t="s" s="6">
-        <v>766</v>
       </c>
       <c r="C4" t="s" s="3">
         <v>447</v>
       </c>
       <c r="D4" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E4" s="4"/>
     </row>
     <row r="5" ht="13.65" customHeight="1">
       <c r="A5" t="s" s="3">
+        <v>767</v>
+      </c>
+      <c r="B5" t="s" s="3">
         <v>768</v>
-      </c>
-      <c r="B5" t="s" s="3">
-        <v>769</v>
       </c>
       <c r="C5" t="s" s="3">
         <v>447</v>
       </c>
       <c r="D5" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E5" s="4"/>
     </row>
@@ -19444,13 +19441,13 @@
         <v>614</v>
       </c>
       <c r="B6" t="s" s="7">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C6" t="s" s="7">
         <v>447</v>
       </c>
       <c r="D6" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E6" s="4"/>
     </row>
@@ -19459,88 +19456,88 @@
         <v>614</v>
       </c>
       <c r="B7" t="s" s="3">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C7" t="s" s="3">
         <v>447</v>
       </c>
       <c r="D7" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E7" s="4"/>
     </row>
     <row r="8" ht="13.65" customHeight="1">
       <c r="A8" t="s" s="7">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="B8" t="s" s="7">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="C8" t="s" s="7">
         <v>447</v>
       </c>
       <c r="D8" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E8" s="4"/>
     </row>
     <row r="9" ht="13.65" customHeight="1">
       <c r="A9" t="s" s="7">
+        <v>767</v>
+      </c>
+      <c r="B9" t="s" s="7">
         <v>768</v>
-      </c>
-      <c r="B9" t="s" s="7">
-        <v>769</v>
       </c>
       <c r="C9" t="s" s="7">
         <v>447</v>
       </c>
       <c r="D9" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E9" s="4"/>
     </row>
     <row r="10" ht="13.65" customHeight="1">
       <c r="A10" t="s" s="6">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B10" t="s" s="3">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="C10" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D10" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E10" s="4"/>
     </row>
     <row r="11" ht="13.65" customHeight="1">
       <c r="A11" t="s" s="3">
+        <v>773</v>
+      </c>
+      <c r="B11" t="s" s="3">
         <v>774</v>
       </c>
-      <c r="B11" t="s" s="3">
-        <v>775</v>
-      </c>
       <c r="C11" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D11" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E11" s="4"/>
     </row>
     <row r="12" ht="13.65" customHeight="1">
       <c r="A12" t="s" s="3">
+        <v>775</v>
+      </c>
+      <c r="B12" t="s" s="3">
         <v>776</v>
       </c>
-      <c r="B12" t="s" s="3">
-        <v>777</v>
-      </c>
       <c r="C12" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D12" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E12" s="4"/>
     </row>
@@ -19549,13 +19546,13 @@
         <v>620</v>
       </c>
       <c r="B13" t="s" s="3">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C13" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D13" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E13" s="4"/>
     </row>
@@ -19564,43 +19561,43 @@
         <v>451</v>
       </c>
       <c r="B14" t="s" s="3">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C14" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D14" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E14" s="4"/>
     </row>
     <row r="15" ht="13.65" customHeight="1">
       <c r="A15" t="s" s="3">
+        <v>779</v>
+      </c>
+      <c r="B15" t="s" s="3">
         <v>780</v>
       </c>
-      <c r="B15" t="s" s="3">
-        <v>781</v>
-      </c>
       <c r="C15" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D15" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E15" s="4"/>
     </row>
     <row r="16" ht="13.65" customHeight="1">
       <c r="A16" t="s" s="3">
+        <v>781</v>
+      </c>
+      <c r="B16" t="s" s="3">
         <v>782</v>
       </c>
-      <c r="B16" t="s" s="3">
-        <v>783</v>
-      </c>
       <c r="C16" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D16" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E16" s="4"/>
     </row>
@@ -19609,13 +19606,13 @@
         <v>520</v>
       </c>
       <c r="B17" t="s" s="3">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="C17" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D17" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E17" s="4"/>
     </row>
@@ -19624,43 +19621,43 @@
         <v>546</v>
       </c>
       <c r="B18" t="s" s="3">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C18" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D18" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E18" s="4"/>
     </row>
     <row r="19" ht="13.65" customHeight="1">
       <c r="A19" t="s" s="3">
+        <v>785</v>
+      </c>
+      <c r="B19" t="s" s="3">
         <v>786</v>
       </c>
-      <c r="B19" t="s" s="3">
-        <v>787</v>
-      </c>
       <c r="C19" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D19" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E19" s="4"/>
     </row>
     <row r="20" ht="13.65" customHeight="1">
       <c r="A20" t="s" s="7">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B20" t="s" s="7">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="C20" t="s" s="7">
         <v>178</v>
       </c>
       <c r="D20" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E20" s="4"/>
     </row>
@@ -19669,13 +19666,13 @@
         <v>668</v>
       </c>
       <c r="B21" t="s" s="3">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="C21" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D21" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E21" s="4"/>
     </row>
@@ -19684,133 +19681,133 @@
         <v>727</v>
       </c>
       <c r="B22" t="s" s="3">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="C22" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D22" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E22" s="4"/>
     </row>
     <row r="23" ht="13.65" customHeight="1">
       <c r="A23" t="s" s="3">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B23" t="s" s="3">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="C23" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D23" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E23" s="4"/>
     </row>
     <row r="24" ht="13.65" customHeight="1">
       <c r="A24" t="s" s="7">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B24" t="s" s="7">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="C24" t="s" s="7">
         <v>178</v>
       </c>
       <c r="D24" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E24" s="4"/>
     </row>
     <row r="25" ht="13.65" customHeight="1">
       <c r="A25" t="s" s="8">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B25" t="s" s="8">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="C25" t="s" s="8">
         <v>178</v>
       </c>
       <c r="D25" t="s" s="8">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E25" s="4"/>
     </row>
     <row r="26" ht="13.65" customHeight="1">
       <c r="A26" t="s" s="3">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B26" t="s" s="3">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="C26" t="s" s="3">
         <v>178</v>
       </c>
       <c r="D26" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E26" s="4"/>
     </row>
     <row r="27" ht="13.65" customHeight="1">
       <c r="A27" t="s" s="7">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B27" t="s" s="7">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="C27" t="s" s="7">
         <v>178</v>
       </c>
       <c r="D27" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E27" s="4"/>
     </row>
     <row r="28" ht="13.65" customHeight="1">
       <c r="A28" t="s" s="3">
+        <v>794</v>
+      </c>
+      <c r="B28" t="s" s="3">
         <v>795</v>
-      </c>
-      <c r="B28" t="s" s="3">
-        <v>796</v>
       </c>
       <c r="C28" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D28" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E28" s="4"/>
     </row>
     <row r="29" ht="13.65" customHeight="1">
       <c r="A29" t="s" s="3">
+        <v>796</v>
+      </c>
+      <c r="B29" t="s" s="3">
         <v>797</v>
-      </c>
-      <c r="B29" t="s" s="3">
-        <v>798</v>
       </c>
       <c r="C29" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D29" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E29" s="4"/>
     </row>
     <row r="30" ht="13.65" customHeight="1">
       <c r="A30" t="s" s="3">
+        <v>798</v>
+      </c>
+      <c r="B30" t="s" s="3">
         <v>799</v>
-      </c>
-      <c r="B30" t="s" s="3">
-        <v>800</v>
       </c>
       <c r="C30" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D30" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E30" s="4"/>
     </row>
@@ -19819,13 +19816,13 @@
         <v>624</v>
       </c>
       <c r="B31" t="s" s="6">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="C31" t="s" s="6">
         <v>514</v>
       </c>
       <c r="D31" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E31" s="4"/>
     </row>
@@ -19834,28 +19831,28 @@
         <v>705</v>
       </c>
       <c r="B32" t="s" s="3">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="C32" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D32" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E32" s="4"/>
     </row>
     <row r="33" ht="13.65" customHeight="1">
       <c r="A33" t="s" s="3">
+        <v>802</v>
+      </c>
+      <c r="B33" t="s" s="3">
         <v>803</v>
-      </c>
-      <c r="B33" t="s" s="3">
-        <v>804</v>
       </c>
       <c r="C33" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D33" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E33" s="4"/>
     </row>
@@ -19864,28 +19861,28 @@
         <v>619</v>
       </c>
       <c r="B34" t="s" s="3">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="C34" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D34" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E34" s="4"/>
     </row>
     <row r="35" ht="13.65" customHeight="1">
       <c r="A35" t="s" s="3">
+        <v>805</v>
+      </c>
+      <c r="B35" t="s" s="3">
         <v>806</v>
-      </c>
-      <c r="B35" t="s" s="3">
-        <v>807</v>
       </c>
       <c r="C35" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D35" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E35" s="4"/>
     </row>
@@ -19894,28 +19891,28 @@
         <v>513</v>
       </c>
       <c r="B36" t="s" s="3">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="C36" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D36" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E36" s="4"/>
     </row>
     <row r="37" ht="13.65" customHeight="1">
       <c r="A37" t="s" s="7">
+        <v>808</v>
+      </c>
+      <c r="B37" t="s" s="7">
         <v>809</v>
-      </c>
-      <c r="B37" t="s" s="7">
-        <v>810</v>
       </c>
       <c r="C37" t="s" s="7">
         <v>514</v>
       </c>
       <c r="D37" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E37" s="4"/>
     </row>
@@ -19924,13 +19921,13 @@
         <v>576</v>
       </c>
       <c r="B38" t="s" s="3">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="C38" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D38" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E38" s="4"/>
     </row>
@@ -19939,13 +19936,13 @@
         <v>624</v>
       </c>
       <c r="B39" t="s" s="7">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="C39" t="s" s="7">
         <v>514</v>
       </c>
       <c r="D39" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E39" s="4"/>
     </row>
@@ -19954,13 +19951,13 @@
         <v>699</v>
       </c>
       <c r="B40" t="s" s="3">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="C40" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D40" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E40" s="4"/>
     </row>
@@ -19969,118 +19966,118 @@
         <v>705</v>
       </c>
       <c r="B41" t="s" s="7">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="C41" t="s" s="7">
         <v>514</v>
       </c>
       <c r="D41" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E41" s="4"/>
     </row>
     <row r="42" ht="13.65" customHeight="1">
       <c r="A42" t="s" s="7">
+        <v>802</v>
+      </c>
+      <c r="B42" t="s" s="7">
         <v>803</v>
-      </c>
-      <c r="B42" t="s" s="7">
-        <v>804</v>
       </c>
       <c r="C42" t="s" s="7">
         <v>514</v>
       </c>
       <c r="D42" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E42" s="4"/>
     </row>
     <row r="43" ht="13.65" customHeight="1">
       <c r="A43" t="s" s="6">
+        <v>814</v>
+      </c>
+      <c r="B43" t="s" s="6">
         <v>815</v>
-      </c>
-      <c r="B43" t="s" s="6">
-        <v>816</v>
       </c>
       <c r="C43" t="s" s="6">
         <v>514</v>
       </c>
       <c r="D43" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E43" s="4"/>
     </row>
     <row r="44" ht="13.65" customHeight="1">
       <c r="A44" t="s" s="3">
+        <v>816</v>
+      </c>
+      <c r="B44" t="s" s="3">
         <v>817</v>
-      </c>
-      <c r="B44" t="s" s="3">
-        <v>818</v>
       </c>
       <c r="C44" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D44" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E44" s="4"/>
     </row>
     <row r="45" ht="13.65" customHeight="1">
       <c r="A45" t="s" s="3">
+        <v>818</v>
+      </c>
+      <c r="B45" t="s" s="3">
         <v>819</v>
-      </c>
-      <c r="B45" t="s" s="3">
-        <v>820</v>
       </c>
       <c r="C45" t="s" s="3">
         <v>514</v>
       </c>
       <c r="D45" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E45" s="4"/>
     </row>
     <row r="46" ht="13.65" customHeight="1">
       <c r="A46" t="s" s="7">
+        <v>820</v>
+      </c>
+      <c r="B46" t="s" s="7">
         <v>821</v>
-      </c>
-      <c r="B46" t="s" s="7">
-        <v>822</v>
       </c>
       <c r="C46" t="s" s="7">
         <v>514</v>
       </c>
       <c r="D46" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E46" s="4"/>
     </row>
     <row r="47" ht="13.65" customHeight="1">
       <c r="A47" t="s" s="7">
+        <v>816</v>
+      </c>
+      <c r="B47" t="s" s="7">
         <v>817</v>
-      </c>
-      <c r="B47" t="s" s="7">
-        <v>818</v>
       </c>
       <c r="C47" t="s" s="7">
         <v>514</v>
       </c>
       <c r="D47" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E47" s="4"/>
     </row>
     <row r="48" ht="13.65" customHeight="1">
       <c r="A48" t="s" s="3">
+        <v>822</v>
+      </c>
+      <c r="B48" t="s" s="3">
         <v>823</v>
       </c>
-      <c r="B48" t="s" s="3">
-        <v>824</v>
-      </c>
       <c r="C48" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D48" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E48" s="4"/>
     </row>
@@ -20089,43 +20086,43 @@
         <v>346</v>
       </c>
       <c r="B49" t="s" s="3">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="C49" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D49" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E49" s="4"/>
     </row>
     <row r="50" ht="13.65" customHeight="1">
       <c r="A50" t="s" s="3">
+        <v>825</v>
+      </c>
+      <c r="B50" t="s" s="3">
         <v>826</v>
       </c>
-      <c r="B50" t="s" s="3">
-        <v>827</v>
-      </c>
       <c r="C50" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D50" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E50" s="4"/>
     </row>
     <row r="51" ht="13.65" customHeight="1">
       <c r="A51" t="s" s="3">
+        <v>827</v>
+      </c>
+      <c r="B51" t="s" s="3">
         <v>828</v>
       </c>
-      <c r="B51" t="s" s="3">
-        <v>829</v>
-      </c>
       <c r="C51" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D51" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E51" s="4"/>
     </row>
@@ -20134,13 +20131,13 @@
         <v>459</v>
       </c>
       <c r="B52" t="s" s="3">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="C52" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D52" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E52" s="4"/>
     </row>
@@ -20149,13 +20146,13 @@
         <v>544</v>
       </c>
       <c r="B53" t="s" s="3">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="C53" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D53" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E53" s="4"/>
     </row>
@@ -20164,13 +20161,13 @@
         <v>617</v>
       </c>
       <c r="B54" t="s" s="3">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="C54" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D54" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E54" s="4"/>
     </row>
@@ -20179,13 +20176,13 @@
         <v>622</v>
       </c>
       <c r="B55" t="s" s="3">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="C55" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D55" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E55" s="4"/>
     </row>
@@ -20194,13 +20191,13 @@
         <v>623</v>
       </c>
       <c r="B56" t="s" s="3">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="C56" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D56" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E56" s="4"/>
     </row>
@@ -20209,13 +20206,13 @@
         <v>665</v>
       </c>
       <c r="B57" t="s" s="6">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="C57" t="s" s="6">
         <v>347</v>
       </c>
       <c r="D57" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E57" s="4"/>
     </row>
@@ -20224,13 +20221,13 @@
         <v>631</v>
       </c>
       <c r="B58" t="s" s="6">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C58" t="s" s="6">
         <v>347</v>
       </c>
       <c r="D58" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E58" s="4"/>
     </row>
@@ -20239,58 +20236,58 @@
         <v>667</v>
       </c>
       <c r="B59" t="s" s="6">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="C59" t="s" s="6">
         <v>347</v>
       </c>
       <c r="D59" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E59" s="4"/>
     </row>
     <row r="60" ht="13.65" customHeight="1">
       <c r="A60" t="s" s="6">
+        <v>837</v>
+      </c>
+      <c r="B60" t="s" s="6">
         <v>838</v>
       </c>
-      <c r="B60" t="s" s="6">
-        <v>839</v>
-      </c>
       <c r="C60" t="s" s="6">
         <v>347</v>
       </c>
       <c r="D60" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E60" s="4"/>
     </row>
     <row r="61" ht="13.65" customHeight="1">
       <c r="A61" t="s" s="6">
+        <v>839</v>
+      </c>
+      <c r="B61" t="s" s="3">
         <v>840</v>
       </c>
-      <c r="B61" t="s" s="3">
-        <v>841</v>
-      </c>
       <c r="C61" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D61" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E61" s="4"/>
     </row>
     <row r="62" ht="13.65" customHeight="1">
       <c r="A62" t="s" s="6">
+        <v>841</v>
+      </c>
+      <c r="B62" t="s" s="6">
         <v>842</v>
       </c>
-      <c r="B62" t="s" s="6">
-        <v>843</v>
-      </c>
       <c r="C62" t="s" s="6">
         <v>347</v>
       </c>
       <c r="D62" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E62" s="4"/>
     </row>
@@ -20299,13 +20296,13 @@
         <v>711</v>
       </c>
       <c r="B63" t="s" s="3">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="C63" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D63" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E63" s="4"/>
     </row>
@@ -20314,28 +20311,28 @@
         <v>696</v>
       </c>
       <c r="B64" t="s" s="3">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="C64" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D64" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E64" s="4"/>
     </row>
     <row r="65" ht="13.65" customHeight="1">
       <c r="A65" t="s" s="3">
+        <v>845</v>
+      </c>
+      <c r="B65" t="s" s="3">
         <v>846</v>
       </c>
-      <c r="B65" t="s" s="3">
-        <v>847</v>
-      </c>
       <c r="C65" t="s" s="3">
         <v>347</v>
       </c>
       <c r="D65" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E65" s="4"/>
     </row>
@@ -20344,13 +20341,13 @@
         <v>696</v>
       </c>
       <c r="B66" t="s" s="7">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="C66" t="s" s="7">
         <v>347</v>
       </c>
       <c r="D66" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E66" s="4"/>
     </row>
@@ -20359,13 +20356,13 @@
         <v>711</v>
       </c>
       <c r="B67" t="s" s="7">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="C67" t="s" s="7">
         <v>347</v>
       </c>
       <c r="D67" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E67" s="4"/>
     </row>
@@ -20374,28 +20371,28 @@
         <v>574</v>
       </c>
       <c r="B68" t="s" s="3">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="C68" t="s" s="3">
         <v>457</v>
       </c>
       <c r="D68" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E68" s="4"/>
     </row>
     <row r="69" ht="13.65" customHeight="1">
       <c r="A69" t="s" s="6">
+        <v>850</v>
+      </c>
+      <c r="B69" t="s" s="6">
         <v>851</v>
       </c>
-      <c r="B69" t="s" s="6">
+      <c r="C69" t="s" s="6">
         <v>852</v>
       </c>
-      <c r="C69" t="s" s="6">
-        <v>853</v>
-      </c>
       <c r="D69" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E69" s="4"/>
     </row>
@@ -20404,118 +20401,118 @@
         <v>456</v>
       </c>
       <c r="B70" t="s" s="3">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="C70" t="s" s="3">
         <v>457</v>
       </c>
       <c r="D70" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E70" s="4"/>
     </row>
     <row r="71" ht="13.65" customHeight="1">
       <c r="A71" t="s" s="3">
+        <v>854</v>
+      </c>
+      <c r="B71" t="s" s="3">
         <v>855</v>
-      </c>
-      <c r="B71" t="s" s="3">
-        <v>856</v>
       </c>
       <c r="C71" t="s" s="3">
         <v>457</v>
       </c>
       <c r="D71" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E71" s="4"/>
     </row>
     <row r="72" ht="13.65" customHeight="1">
       <c r="A72" t="s" s="3">
+        <v>856</v>
+      </c>
+      <c r="B72" t="s" s="3">
         <v>857</v>
-      </c>
-      <c r="B72" t="s" s="3">
-        <v>858</v>
       </c>
       <c r="C72" t="s" s="3">
         <v>457</v>
       </c>
       <c r="D72" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E72" s="4"/>
     </row>
     <row r="73" ht="13.65" customHeight="1">
       <c r="A73" t="s" s="3">
+        <v>858</v>
+      </c>
+      <c r="B73" t="s" s="3">
         <v>859</v>
-      </c>
-      <c r="B73" t="s" s="3">
-        <v>860</v>
       </c>
       <c r="C73" t="s" s="3">
         <v>457</v>
       </c>
       <c r="D73" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E73" s="4"/>
     </row>
     <row r="74" ht="13.65" customHeight="1">
       <c r="A74" t="s" s="3">
+        <v>737</v>
+      </c>
+      <c r="B74" t="s" s="3">
+        <v>860</v>
+      </c>
+      <c r="C74" t="s" s="3">
         <v>738</v>
       </c>
-      <c r="B74" t="s" s="3">
-        <v>861</v>
-      </c>
-      <c r="C74" t="s" s="3">
-        <v>739</v>
-      </c>
       <c r="D74" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E74" s="4"/>
     </row>
     <row r="75" ht="13.65" customHeight="1">
       <c r="A75" t="s" s="3">
+        <v>861</v>
+      </c>
+      <c r="B75" t="s" s="3">
         <v>862</v>
       </c>
-      <c r="B75" t="s" s="3">
-        <v>863</v>
-      </c>
       <c r="C75" t="s" s="3">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D75" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E75" s="4"/>
     </row>
     <row r="76" ht="13.65" customHeight="1">
       <c r="A76" t="s" s="3">
+        <v>863</v>
+      </c>
+      <c r="B76" t="s" s="3">
         <v>864</v>
       </c>
-      <c r="B76" t="s" s="3">
-        <v>865</v>
-      </c>
       <c r="C76" t="s" s="3">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D76" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E76" s="4"/>
     </row>
     <row r="77" ht="13.65" customHeight="1">
       <c r="A77" t="s" s="7">
+        <v>737</v>
+      </c>
+      <c r="B77" t="s" s="7">
+        <v>860</v>
+      </c>
+      <c r="C77" t="s" s="7">
         <v>738</v>
       </c>
-      <c r="B77" t="s" s="7">
-        <v>861</v>
-      </c>
-      <c r="C77" t="s" s="7">
-        <v>739</v>
-      </c>
       <c r="D77" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E77" s="4"/>
     </row>
@@ -20524,28 +20521,28 @@
         <v>618</v>
       </c>
       <c r="B78" t="s" s="3">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="C78" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D78" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E78" s="4"/>
     </row>
     <row r="79" ht="13.65" customHeight="1">
       <c r="A79" t="s" s="8">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B79" t="s" s="8">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="C79" t="s" s="8">
         <v>444</v>
       </c>
       <c r="D79" t="s" s="8">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E79" s="4"/>
     </row>
@@ -20554,43 +20551,43 @@
         <v>443</v>
       </c>
       <c r="B80" t="s" s="3">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="C80" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D80" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E80" s="4"/>
     </row>
     <row r="81" ht="13.65" customHeight="1">
       <c r="A81" t="s" s="3">
+        <v>868</v>
+      </c>
+      <c r="B81" t="s" s="3">
         <v>869</v>
-      </c>
-      <c r="B81" t="s" s="3">
-        <v>870</v>
       </c>
       <c r="C81" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D81" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E81" s="4"/>
     </row>
     <row r="82" ht="13.65" customHeight="1">
       <c r="A82" t="s" s="3">
+        <v>870</v>
+      </c>
+      <c r="B82" t="s" s="3">
         <v>871</v>
-      </c>
-      <c r="B82" t="s" s="3">
-        <v>872</v>
       </c>
       <c r="C82" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D82" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E82" s="4"/>
     </row>
@@ -20599,28 +20596,28 @@
         <v>627</v>
       </c>
       <c r="B83" t="s" s="6">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="C83" t="s" s="6">
         <v>444</v>
       </c>
       <c r="D83" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E83" s="4"/>
     </row>
     <row r="84" ht="13.65" customHeight="1">
       <c r="A84" t="s" s="3">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B84" t="s" s="3">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="C84" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D84" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E84" s="4"/>
     </row>
@@ -20629,13 +20626,13 @@
         <v>449</v>
       </c>
       <c r="B85" t="s" s="3">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="C85" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D85" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E85" s="4"/>
     </row>
@@ -20644,43 +20641,43 @@
         <v>454</v>
       </c>
       <c r="B86" t="s" s="3">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="C86" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D86" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E86" s="4"/>
     </row>
     <row r="87" ht="13.65" customHeight="1">
       <c r="A87" t="s" s="3">
+        <v>876</v>
+      </c>
+      <c r="B87" t="s" s="3">
         <v>877</v>
-      </c>
-      <c r="B87" t="s" s="3">
-        <v>878</v>
       </c>
       <c r="C87" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D87" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E87" s="4"/>
     </row>
     <row r="88" ht="13.65" customHeight="1">
       <c r="A88" t="s" s="3">
+        <v>878</v>
+      </c>
+      <c r="B88" t="s" s="3">
         <v>879</v>
-      </c>
-      <c r="B88" t="s" s="3">
-        <v>880</v>
       </c>
       <c r="C88" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D88" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E88" s="4"/>
     </row>
@@ -20689,13 +20686,13 @@
         <v>572</v>
       </c>
       <c r="B89" t="s" s="3">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="C89" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D89" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E89" s="4"/>
     </row>
@@ -20704,13 +20701,13 @@
         <v>555</v>
       </c>
       <c r="B90" t="s" s="3">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="C90" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D90" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E90" s="4"/>
     </row>
@@ -20719,13 +20716,13 @@
         <v>573</v>
       </c>
       <c r="B91" t="s" s="3">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="C91" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D91" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E91" s="4"/>
     </row>
@@ -20734,28 +20731,28 @@
         <v>611</v>
       </c>
       <c r="B92" t="s" s="3">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="C92" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D92" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E92" s="4"/>
     </row>
     <row r="93" ht="13.65" customHeight="1">
       <c r="A93" t="s" s="3">
+        <v>884</v>
+      </c>
+      <c r="B93" t="s" s="3">
         <v>885</v>
-      </c>
-      <c r="B93" t="s" s="3">
-        <v>886</v>
       </c>
       <c r="C93" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D93" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E93" s="4"/>
     </row>
@@ -20764,13 +20761,13 @@
         <v>629</v>
       </c>
       <c r="B94" t="s" s="6">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="C94" t="s" s="6">
         <v>444</v>
       </c>
       <c r="D94" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E94" s="4"/>
     </row>
@@ -20779,58 +20776,58 @@
         <v>663</v>
       </c>
       <c r="B95" t="s" s="6">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C95" t="s" s="6">
         <v>444</v>
       </c>
       <c r="D95" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E95" s="4"/>
     </row>
     <row r="96" ht="13.65" customHeight="1">
       <c r="A96" t="s" s="3">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B96" t="s" s="3">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="C96" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D96" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E96" s="4"/>
     </row>
     <row r="97" ht="13.65" customHeight="1">
       <c r="A97" t="s" s="3">
+        <v>889</v>
+      </c>
+      <c r="B97" t="s" s="3">
         <v>890</v>
-      </c>
-      <c r="B97" t="s" s="3">
-        <v>891</v>
       </c>
       <c r="C97" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D97" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E97" s="4"/>
     </row>
     <row r="98" ht="13.65" customHeight="1">
       <c r="A98" t="s" s="3">
+        <v>891</v>
+      </c>
+      <c r="B98" t="s" s="3">
         <v>892</v>
-      </c>
-      <c r="B98" t="s" s="3">
-        <v>893</v>
       </c>
       <c r="C98" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D98" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E98" s="4"/>
     </row>
@@ -20839,88 +20836,88 @@
         <v>729</v>
       </c>
       <c r="B99" t="s" s="3">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="C99" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D99" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E99" s="4"/>
     </row>
     <row r="100" ht="13.65" customHeight="1">
       <c r="A100" t="s" s="7">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B100" t="s" s="7">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="C100" t="s" s="7">
         <v>444</v>
       </c>
       <c r="D100" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E100" s="4"/>
     </row>
     <row r="101" ht="13.65" customHeight="1">
       <c r="A101" t="s" s="3">
+        <v>895</v>
+      </c>
+      <c r="B101" t="s" s="3">
         <v>896</v>
-      </c>
-      <c r="B101" t="s" s="3">
-        <v>897</v>
       </c>
       <c r="C101" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D101" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E101" s="4"/>
     </row>
     <row r="102" ht="13.65" customHeight="1">
       <c r="A102" t="s" s="3">
+        <v>897</v>
+      </c>
+      <c r="B102" t="s" s="3">
         <v>898</v>
-      </c>
-      <c r="B102" t="s" s="3">
-        <v>899</v>
       </c>
       <c r="C102" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D102" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E102" s="4"/>
     </row>
     <row r="103" ht="13.65" customHeight="1">
       <c r="A103" t="s" s="3">
+        <v>899</v>
+      </c>
+      <c r="B103" t="s" s="3">
         <v>900</v>
-      </c>
-      <c r="B103" t="s" s="3">
-        <v>901</v>
       </c>
       <c r="C103" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D103" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E103" s="4"/>
     </row>
     <row r="104" ht="13.65" customHeight="1">
       <c r="A104" t="s" s="3">
+        <v>901</v>
+      </c>
+      <c r="B104" t="s" s="3">
         <v>902</v>
-      </c>
-      <c r="B104" t="s" s="3">
-        <v>903</v>
       </c>
       <c r="C104" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D104" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E104" s="4"/>
     </row>
@@ -20929,13 +20926,13 @@
         <v>523</v>
       </c>
       <c r="B105" t="s" s="3">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="C105" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D105" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E105" s="4"/>
     </row>
@@ -20944,208 +20941,208 @@
         <v>730</v>
       </c>
       <c r="B106" t="s" s="3">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="C106" t="s" s="3">
         <v>444</v>
       </c>
       <c r="D106" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E106" s="4"/>
     </row>
     <row r="107" ht="13.65" customHeight="1">
       <c r="A107" t="s" s="7">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B107" t="s" s="7">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="C107" t="s" s="7">
         <v>444</v>
       </c>
       <c r="D107" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E107" s="4"/>
     </row>
     <row r="108" ht="13.65" customHeight="1">
       <c r="A108" t="s" s="3">
+        <v>906</v>
+      </c>
+      <c r="B108" t="s" s="3">
         <v>907</v>
-      </c>
-      <c r="B108" t="s" s="3">
-        <v>908</v>
       </c>
       <c r="C108" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D108" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E108" s="4"/>
     </row>
     <row r="109" ht="13.65" customHeight="1">
       <c r="A109" t="s" s="6">
+        <v>908</v>
+      </c>
+      <c r="B109" t="s" s="3">
         <v>909</v>
-      </c>
-      <c r="B109" t="s" s="3">
-        <v>910</v>
       </c>
       <c r="C109" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D109" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E109" s="4"/>
     </row>
     <row r="110" ht="13.65" customHeight="1">
       <c r="A110" t="s" s="7">
+        <v>910</v>
+      </c>
+      <c r="B110" t="s" s="7">
         <v>911</v>
-      </c>
-      <c r="B110" t="s" s="7">
-        <v>912</v>
       </c>
       <c r="C110" t="s" s="7">
         <v>7</v>
       </c>
       <c r="D110" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E110" s="4"/>
     </row>
     <row r="111" ht="13.65" customHeight="1">
       <c r="A111" t="s" s="3">
+        <v>912</v>
+      </c>
+      <c r="B111" t="s" s="3">
         <v>913</v>
-      </c>
-      <c r="B111" t="s" s="3">
-        <v>914</v>
       </c>
       <c r="C111" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D111" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E111" s="4"/>
     </row>
     <row r="112" ht="13.65" customHeight="1">
       <c r="A112" t="s" s="3">
+        <v>914</v>
+      </c>
+      <c r="B112" t="s" s="3">
         <v>915</v>
-      </c>
-      <c r="B112" t="s" s="3">
-        <v>916</v>
       </c>
       <c r="C112" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D112" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E112" s="4"/>
     </row>
     <row r="113" ht="13.65" customHeight="1">
       <c r="A113" t="s" s="3">
+        <v>916</v>
+      </c>
+      <c r="B113" t="s" s="3">
         <v>917</v>
-      </c>
-      <c r="B113" t="s" s="3">
-        <v>918</v>
       </c>
       <c r="C113" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D113" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E113" s="4"/>
     </row>
     <row r="114" ht="13.65" customHeight="1">
       <c r="A114" t="s" s="7">
+        <v>906</v>
+      </c>
+      <c r="B114" t="s" s="7">
         <v>907</v>
-      </c>
-      <c r="B114" t="s" s="7">
-        <v>908</v>
       </c>
       <c r="C114" t="s" s="7">
         <v>7</v>
       </c>
       <c r="D114" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E114" s="4"/>
     </row>
     <row r="115" ht="13.65" customHeight="1">
       <c r="A115" t="s" s="3">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="B115" t="s" s="3">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="C115" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D115" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E115" s="4"/>
     </row>
     <row r="116" ht="13.65" customHeight="1">
       <c r="A116" t="s" s="3">
+        <v>919</v>
+      </c>
+      <c r="B116" t="s" s="3">
         <v>920</v>
-      </c>
-      <c r="B116" t="s" s="3">
-        <v>921</v>
       </c>
       <c r="C116" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D116" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E116" s="4"/>
     </row>
     <row r="117" ht="13.65" customHeight="1">
       <c r="A117" t="s" s="3">
+        <v>921</v>
+      </c>
+      <c r="B117" t="s" s="3">
         <v>922</v>
-      </c>
-      <c r="B117" t="s" s="3">
-        <v>923</v>
       </c>
       <c r="C117" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D117" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E117" s="4"/>
     </row>
     <row r="118" ht="13.65" customHeight="1">
       <c r="A118" t="s" s="6">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B118" t="s" s="6">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="C118" t="s" s="6">
         <v>7</v>
       </c>
       <c r="D118" t="s" s="6">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E118" s="4"/>
     </row>
     <row r="119" ht="13.65" customHeight="1">
       <c r="A119" t="s" s="7">
+        <v>924</v>
+      </c>
+      <c r="B119" t="s" s="7">
         <v>925</v>
-      </c>
-      <c r="B119" t="s" s="7">
-        <v>926</v>
       </c>
       <c r="C119" t="s" s="7">
         <v>7</v>
       </c>
       <c r="D119" t="s" s="7">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E119" s="4"/>
     </row>
@@ -21154,13 +21151,13 @@
         <v>701</v>
       </c>
       <c r="B120" t="s" s="3">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="C120" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D120" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E120" s="4"/>
     </row>
@@ -21169,13 +21166,13 @@
         <v>703</v>
       </c>
       <c r="B121" t="s" s="3">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="C121" t="s" s="3">
         <v>7</v>
       </c>
       <c r="D121" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E121" s="4"/>
     </row>
@@ -21184,13 +21181,13 @@
         <v>446</v>
       </c>
       <c r="B122" t="s" s="3">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="C122" t="s" s="3">
         <v>447</v>
       </c>
       <c r="D122" t="s" s="3">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="E122" s="4"/>
     </row>
@@ -21217,13 +21214,13 @@
   <sheetData>
     <row r="1" ht="13.65" customHeight="1">
       <c r="A1" t="s" s="2">
+        <v>929</v>
+      </c>
+      <c r="B1" t="s" s="2">
         <v>930</v>
       </c>
-      <c r="B1" t="s" s="2">
+      <c r="C1" t="s" s="2">
         <v>931</v>
-      </c>
-      <c r="C1" t="s" s="2">
-        <v>932</v>
       </c>
       <c r="D1" s="10"/>
       <c r="E1" s="11"/>
@@ -21233,10 +21230,10 @@
         <v>13</v>
       </c>
       <c r="B2" t="s" s="3">
+        <v>932</v>
+      </c>
+      <c r="C2" t="s" s="3">
         <v>933</v>
-      </c>
-      <c r="C2" t="s" s="3">
-        <v>934</v>
       </c>
       <c r="D2" s="12"/>
       <c r="E2" s="13"/>
@@ -21246,10 +21243,10 @@
         <v>86</v>
       </c>
       <c r="B3" t="s" s="3">
+        <v>934</v>
+      </c>
+      <c r="C3" t="s" s="3">
         <v>935</v>
-      </c>
-      <c r="C3" t="s" s="3">
-        <v>936</v>
       </c>
       <c r="D3" s="12"/>
       <c r="E3" s="13"/>
@@ -21259,10 +21256,10 @@
         <v>14</v>
       </c>
       <c r="B4" t="s" s="3">
+        <v>936</v>
+      </c>
+      <c r="C4" t="s" s="3">
         <v>937</v>
-      </c>
-      <c r="C4" t="s" s="3">
-        <v>938</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="13"/>
@@ -21272,23 +21269,23 @@
         <v>10</v>
       </c>
       <c r="B5" t="s" s="3">
+        <v>938</v>
+      </c>
+      <c r="C5" t="s" s="3">
         <v>939</v>
-      </c>
-      <c r="C5" t="s" s="3">
-        <v>940</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="13"/>
     </row>
     <row r="6" ht="13.65" customHeight="1">
       <c r="A6" t="s" s="3">
+        <v>940</v>
+      </c>
+      <c r="B6" t="s" s="3">
         <v>941</v>
       </c>
-      <c r="B6" t="s" s="3">
+      <c r="C6" t="s" s="3">
         <v>942</v>
-      </c>
-      <c r="C6" t="s" s="3">
-        <v>943</v>
       </c>
       <c r="D6" s="12"/>
       <c r="E6" s="13"/>
@@ -21298,10 +21295,10 @@
         <v>17</v>
       </c>
       <c r="B7" t="s" s="3">
+        <v>943</v>
+      </c>
+      <c r="C7" t="s" s="3">
         <v>944</v>
-      </c>
-      <c r="C7" t="s" s="3">
-        <v>945</v>
       </c>
       <c r="D7" s="12"/>
       <c r="E7" s="13"/>
@@ -21311,10 +21308,10 @@
         <v>33</v>
       </c>
       <c r="B8" t="s" s="3">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="C8" t="s" s="3">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="13"/>
@@ -21324,23 +21321,23 @@
         <v>19</v>
       </c>
       <c r="B9" t="s" s="3">
+        <v>946</v>
+      </c>
+      <c r="C9" t="s" s="3">
         <v>947</v>
-      </c>
-      <c r="C9" t="s" s="3">
-        <v>948</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="13"/>
     </row>
     <row r="10" ht="13.65" customHeight="1">
       <c r="A10" t="s" s="3">
+        <v>948</v>
+      </c>
+      <c r="B10" t="s" s="3">
         <v>949</v>
       </c>
-      <c r="B10" t="s" s="3">
+      <c r="C10" t="s" s="3">
         <v>950</v>
-      </c>
-      <c r="C10" t="s" s="3">
-        <v>951</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="13"/>
@@ -21350,49 +21347,49 @@
         <v>132</v>
       </c>
       <c r="B11" t="s" s="3">
+        <v>951</v>
+      </c>
+      <c r="C11" t="s" s="3">
         <v>952</v>
-      </c>
-      <c r="C11" t="s" s="3">
-        <v>953</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="13"/>
     </row>
     <row r="12" ht="13.65" customHeight="1">
       <c r="A12" t="s" s="3">
+        <v>953</v>
+      </c>
+      <c r="B12" t="s" s="3">
         <v>954</v>
       </c>
-      <c r="B12" t="s" s="3">
+      <c r="C12" t="s" s="3">
         <v>955</v>
-      </c>
-      <c r="C12" t="s" s="3">
-        <v>956</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="13"/>
     </row>
     <row r="13" ht="13.65" customHeight="1">
       <c r="A13" t="s" s="3">
+        <v>956</v>
+      </c>
+      <c r="B13" t="s" s="3">
         <v>957</v>
       </c>
-      <c r="B13" t="s" s="3">
+      <c r="C13" t="s" s="3">
         <v>958</v>
-      </c>
-      <c r="C13" t="s" s="3">
-        <v>959</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="13"/>
     </row>
     <row r="14" ht="13.65" customHeight="1">
       <c r="A14" t="s" s="3">
+        <v>959</v>
+      </c>
+      <c r="B14" t="s" s="3">
         <v>960</v>
       </c>
-      <c r="B14" t="s" s="3">
-        <v>961</v>
-      </c>
       <c r="C14" t="s" s="3">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="13"/>
@@ -21402,10 +21399,10 @@
         <v>150</v>
       </c>
       <c r="B15" t="s" s="3">
+        <v>961</v>
+      </c>
+      <c r="C15" t="s" s="3">
         <v>962</v>
-      </c>
-      <c r="C15" t="s" s="3">
-        <v>963</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="13"/>
@@ -21415,10 +21412,10 @@
         <v>25</v>
       </c>
       <c r="B16" t="s" s="3">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="C16" t="s" s="3">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="13"/>
@@ -21428,10 +21425,10 @@
         <v>27</v>
       </c>
       <c r="B17" t="s" s="3">
+        <v>964</v>
+      </c>
+      <c r="C17" t="s" s="3">
         <v>965</v>
-      </c>
-      <c r="C17" t="s" s="3">
-        <v>966</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -21441,23 +21438,23 @@
         <v>198</v>
       </c>
       <c r="B18" t="s" s="3">
+        <v>966</v>
+      </c>
+      <c r="C18" t="s" s="3">
         <v>967</v>
-      </c>
-      <c r="C18" t="s" s="3">
-        <v>968</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="13"/>
     </row>
     <row r="19" ht="13.65" customHeight="1">
       <c r="A19" t="s" s="3">
+        <v>968</v>
+      </c>
+      <c r="B19" t="s" s="3">
         <v>969</v>
       </c>
-      <c r="B19" t="s" s="3">
+      <c r="C19" t="s" s="3">
         <v>970</v>
-      </c>
-      <c r="C19" t="s" s="3">
-        <v>971</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="13"/>
@@ -21467,10 +21464,10 @@
         <v>85</v>
       </c>
       <c r="B20" t="s" s="3">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="C20" t="s" s="3">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="D20" s="12"/>
       <c r="E20" s="13"/>
@@ -21480,23 +21477,23 @@
         <v>126</v>
       </c>
       <c r="B21" t="s" s="3">
+        <v>972</v>
+      </c>
+      <c r="C21" t="s" s="3">
         <v>973</v>
-      </c>
-      <c r="C21" t="s" s="3">
-        <v>974</v>
       </c>
       <c r="D21" s="12"/>
       <c r="E21" s="13"/>
     </row>
     <row r="22" ht="13.65" customHeight="1">
       <c r="A22" t="s" s="3">
+        <v>974</v>
+      </c>
+      <c r="B22" t="s" s="3">
         <v>975</v>
       </c>
-      <c r="B22" t="s" s="3">
+      <c r="C22" t="s" s="3">
         <v>976</v>
-      </c>
-      <c r="C22" t="s" s="3">
-        <v>977</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="13"/>
@@ -21506,10 +21503,10 @@
         <v>99</v>
       </c>
       <c r="B23" t="s" s="3">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="C23" t="s" s="3">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="13"/>
@@ -21519,23 +21516,23 @@
         <v>38</v>
       </c>
       <c r="B24" t="s" s="3">
+        <v>978</v>
+      </c>
+      <c r="C24" t="s" s="3">
         <v>979</v>
-      </c>
-      <c r="C24" t="s" s="3">
-        <v>980</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="13"/>
     </row>
     <row r="25" ht="13.65" customHeight="1">
       <c r="A25" t="s" s="3">
+        <v>980</v>
+      </c>
+      <c r="B25" t="s" s="3">
         <v>981</v>
       </c>
-      <c r="B25" t="s" s="3">
+      <c r="C25" t="s" s="3">
         <v>982</v>
-      </c>
-      <c r="C25" t="s" s="3">
-        <v>983</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="13"/>
@@ -21545,10 +21542,10 @@
         <v>79</v>
       </c>
       <c r="B26" t="s" s="3">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="C26" t="s" s="3">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="13"/>
@@ -21558,75 +21555,75 @@
         <v>155</v>
       </c>
       <c r="B27" t="s" s="3">
+        <v>984</v>
+      </c>
+      <c r="C27" t="s" s="3">
         <v>985</v>
-      </c>
-      <c r="C27" t="s" s="3">
-        <v>986</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="13"/>
     </row>
     <row r="28" ht="13.65" customHeight="1">
       <c r="A28" t="s" s="3">
+        <v>986</v>
+      </c>
+      <c r="B28" t="s" s="3">
         <v>987</v>
       </c>
-      <c r="B28" t="s" s="3">
+      <c r="C28" t="s" s="3">
         <v>988</v>
-      </c>
-      <c r="C28" t="s" s="3">
-        <v>989</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="13"/>
     </row>
     <row r="29" ht="13.65" customHeight="1">
       <c r="A29" t="s" s="3">
+        <v>989</v>
+      </c>
+      <c r="B29" t="s" s="3">
         <v>990</v>
       </c>
-      <c r="B29" t="s" s="3">
+      <c r="C29" t="s" s="3">
         <v>991</v>
-      </c>
-      <c r="C29" t="s" s="3">
-        <v>992</v>
       </c>
       <c r="D29" s="12"/>
       <c r="E29" s="13"/>
     </row>
     <row r="30" ht="13.65" customHeight="1">
       <c r="A30" t="s" s="3">
+        <v>992</v>
+      </c>
+      <c r="B30" t="s" s="3">
         <v>993</v>
       </c>
-      <c r="B30" t="s" s="3">
+      <c r="C30" t="s" s="3">
         <v>994</v>
-      </c>
-      <c r="C30" t="s" s="3">
-        <v>995</v>
       </c>
       <c r="D30" s="12"/>
       <c r="E30" s="13"/>
     </row>
     <row r="31" ht="13.65" customHeight="1">
       <c r="A31" t="s" s="3">
+        <v>995</v>
+      </c>
+      <c r="B31" t="s" s="3">
         <v>996</v>
       </c>
-      <c r="B31" t="s" s="3">
+      <c r="C31" t="s" s="3">
         <v>997</v>
-      </c>
-      <c r="C31" t="s" s="3">
-        <v>998</v>
       </c>
       <c r="D31" s="12"/>
       <c r="E31" s="13"/>
     </row>
     <row r="32" ht="13.65" customHeight="1">
       <c r="A32" t="s" s="3">
+        <v>998</v>
+      </c>
+      <c r="B32" t="s" s="3">
         <v>999</v>
       </c>
-      <c r="B32" t="s" s="3">
+      <c r="C32" t="s" s="3">
         <v>1000</v>
-      </c>
-      <c r="C32" t="s" s="3">
-        <v>1001</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="13"/>
@@ -21636,23 +21633,23 @@
         <v>192</v>
       </c>
       <c r="B33" t="s" s="3">
+        <v>1001</v>
+      </c>
+      <c r="C33" t="s" s="3">
         <v>1002</v>
-      </c>
-      <c r="C33" t="s" s="3">
-        <v>1003</v>
       </c>
       <c r="D33" s="12"/>
       <c r="E33" s="13"/>
     </row>
     <row r="34" ht="13.65" customHeight="1">
       <c r="A34" t="s" s="3">
+        <v>1003</v>
+      </c>
+      <c r="B34" t="s" s="3">
         <v>1004</v>
       </c>
-      <c r="B34" t="s" s="3">
-        <v>1005</v>
-      </c>
       <c r="C34" t="s" s="3">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="13"/>
@@ -21662,10 +21659,10 @@
         <v>87</v>
       </c>
       <c r="B35" t="s" s="3">
+        <v>1005</v>
+      </c>
+      <c r="C35" t="s" s="3">
         <v>1006</v>
-      </c>
-      <c r="C35" t="s" s="3">
-        <v>1007</v>
       </c>
       <c r="D35" s="12"/>
       <c r="E35" s="13"/>
@@ -21675,49 +21672,49 @@
         <v>278</v>
       </c>
       <c r="B36" t="s" s="3">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="C36" t="s" s="3">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="13"/>
     </row>
     <row r="37" ht="13.65" customHeight="1">
       <c r="A37" t="s" s="3">
+        <v>1008</v>
+      </c>
+      <c r="B37" t="s" s="3">
         <v>1009</v>
       </c>
-      <c r="B37" t="s" s="3">
-        <v>1010</v>
-      </c>
       <c r="C37" t="s" s="3">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="D37" s="12"/>
       <c r="E37" s="13"/>
     </row>
     <row r="38" ht="13.65" customHeight="1">
       <c r="A38" t="s" s="3">
+        <v>1010</v>
+      </c>
+      <c r="B38" t="s" s="3">
         <v>1011</v>
       </c>
-      <c r="B38" t="s" s="3">
-        <v>1012</v>
-      </c>
       <c r="C38" t="s" s="3">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="13"/>
     </row>
     <row r="39" ht="13.65" customHeight="1">
       <c r="A39" t="s" s="3">
+        <v>1012</v>
+      </c>
+      <c r="B39" t="s" s="3">
         <v>1013</v>
       </c>
-      <c r="B39" t="s" s="3">
-        <v>1014</v>
-      </c>
       <c r="C39" t="s" s="3">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="D39" s="12"/>
       <c r="E39" s="13"/>
@@ -21727,75 +21724,75 @@
         <v>205</v>
       </c>
       <c r="B40" t="s" s="3">
+        <v>1014</v>
+      </c>
+      <c r="C40" t="s" s="3">
         <v>1015</v>
-      </c>
-      <c r="C40" t="s" s="3">
-        <v>1016</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="13"/>
     </row>
     <row r="41" ht="13.65" customHeight="1">
       <c r="A41" t="s" s="3">
+        <v>1016</v>
+      </c>
+      <c r="B41" t="s" s="3">
         <v>1017</v>
       </c>
-      <c r="B41" t="s" s="3">
+      <c r="C41" t="s" s="3">
         <v>1018</v>
-      </c>
-      <c r="C41" t="s" s="3">
-        <v>1019</v>
       </c>
       <c r="D41" s="12"/>
       <c r="E41" s="13"/>
     </row>
     <row r="42" ht="13.65" customHeight="1">
       <c r="A42" t="s" s="3">
+        <v>1019</v>
+      </c>
+      <c r="B42" t="s" s="3">
         <v>1020</v>
       </c>
-      <c r="B42" t="s" s="3">
+      <c r="C42" t="s" s="3">
         <v>1021</v>
-      </c>
-      <c r="C42" t="s" s="3">
-        <v>1022</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="13"/>
     </row>
     <row r="43" ht="13.65" customHeight="1">
       <c r="A43" t="s" s="3">
+        <v>1022</v>
+      </c>
+      <c r="B43" t="s" s="3">
         <v>1023</v>
       </c>
-      <c r="B43" t="s" s="3">
+      <c r="C43" t="s" s="3">
         <v>1024</v>
-      </c>
-      <c r="C43" t="s" s="3">
-        <v>1025</v>
       </c>
       <c r="D43" s="12"/>
       <c r="E43" s="13"/>
     </row>
     <row r="44" ht="13.65" customHeight="1">
       <c r="A44" t="s" s="3">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="B44" t="s" s="3">
+        <v>1005</v>
+      </c>
+      <c r="C44" t="s" s="3">
         <v>1006</v>
-      </c>
-      <c r="C44" t="s" s="3">
-        <v>1007</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="13"/>
     </row>
     <row r="45" ht="13.65" customHeight="1">
       <c r="A45" t="s" s="3">
+        <v>1026</v>
+      </c>
+      <c r="B45" t="s" s="3">
         <v>1027</v>
       </c>
-      <c r="B45" t="s" s="3">
+      <c r="C45" t="s" s="3">
         <v>1028</v>
-      </c>
-      <c r="C45" t="s" s="3">
-        <v>1029</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="13"/>
@@ -21805,10 +21802,10 @@
         <v>76</v>
       </c>
       <c r="B46" t="s" s="3">
+        <v>1029</v>
+      </c>
+      <c r="C46" t="s" s="3">
         <v>1030</v>
-      </c>
-      <c r="C46" t="s" s="3">
-        <v>1031</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="13"/>
@@ -21818,23 +21815,23 @@
         <v>82</v>
       </c>
       <c r="B47" t="s" s="3">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="C47" t="s" s="3">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="13"/>
     </row>
     <row r="48" ht="13.65" customHeight="1">
       <c r="A48" t="s" s="3">
+        <v>1032</v>
+      </c>
+      <c r="B48" t="s" s="3">
         <v>1033</v>
       </c>
-      <c r="B48" t="s" s="3">
-        <v>1034</v>
-      </c>
       <c r="C48" t="s" s="3">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="13"/>
@@ -21844,49 +21841,49 @@
         <v>90</v>
       </c>
       <c r="B49" t="s" s="3">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="C49" t="s" s="3">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="13"/>
     </row>
     <row r="50" ht="13.65" customHeight="1">
       <c r="A50" t="s" s="3">
+        <v>1035</v>
+      </c>
+      <c r="B50" t="s" s="3">
         <v>1036</v>
       </c>
-      <c r="B50" t="s" s="3">
-        <v>1037</v>
-      </c>
       <c r="C50" t="s" s="3">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="13"/>
     </row>
     <row r="51" ht="13.65" customHeight="1">
       <c r="A51" t="s" s="3">
+        <v>1037</v>
+      </c>
+      <c r="B51" t="s" s="3">
         <v>1038</v>
       </c>
-      <c r="B51" t="s" s="3">
-        <v>1039</v>
-      </c>
       <c r="C51" t="s" s="3">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="13"/>
     </row>
     <row r="52" ht="13.65" customHeight="1">
       <c r="A52" t="s" s="3">
+        <v>1039</v>
+      </c>
+      <c r="B52" t="s" s="3">
         <v>1040</v>
       </c>
-      <c r="B52" t="s" s="3">
+      <c r="C52" t="s" s="3">
         <v>1041</v>
-      </c>
-      <c r="C52" t="s" s="3">
-        <v>1042</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="13"/>
@@ -21896,36 +21893,36 @@
         <v>89</v>
       </c>
       <c r="B53" t="s" s="3">
+        <v>1042</v>
+      </c>
+      <c r="C53" t="s" s="3">
         <v>1043</v>
-      </c>
-      <c r="C53" t="s" s="3">
-        <v>1044</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="13"/>
     </row>
     <row r="54" ht="13.65" customHeight="1">
       <c r="A54" t="s" s="3">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B54" t="s" s="3">
+        <v>946</v>
+      </c>
+      <c r="C54" t="s" s="3">
         <v>947</v>
-      </c>
-      <c r="C54" t="s" s="3">
-        <v>948</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="13"/>
     </row>
     <row r="55" ht="13.65" customHeight="1">
       <c r="A55" t="s" s="3">
+        <v>1045</v>
+      </c>
+      <c r="B55" t="s" s="3">
         <v>1046</v>
       </c>
-      <c r="B55" t="s" s="3">
-        <v>1047</v>
-      </c>
       <c r="C55" t="s" s="3">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="D55" s="12"/>
       <c r="E55" s="13"/>
@@ -21935,23 +21932,23 @@
         <v>97</v>
       </c>
       <c r="B56" t="s" s="3">
+        <v>1047</v>
+      </c>
+      <c r="C56" t="s" s="3">
         <v>1048</v>
-      </c>
-      <c r="C56" t="s" s="3">
-        <v>1049</v>
       </c>
       <c r="D56" s="12"/>
       <c r="E56" s="13"/>
     </row>
     <row r="57" ht="13.65" customHeight="1">
       <c r="A57" t="s" s="3">
+        <v>1049</v>
+      </c>
+      <c r="B57" t="s" s="3">
         <v>1050</v>
       </c>
-      <c r="B57" t="s" s="3">
+      <c r="C57" t="s" s="3">
         <v>1051</v>
-      </c>
-      <c r="C57" t="s" s="3">
-        <v>1052</v>
       </c>
       <c r="D57" s="12"/>
       <c r="E57" s="13"/>
@@ -21961,153 +21958,153 @@
         <v>102</v>
       </c>
       <c r="B58" t="s" s="3">
+        <v>1052</v>
+      </c>
+      <c r="C58" t="s" s="3">
         <v>1053</v>
-      </c>
-      <c r="C58" t="s" s="3">
-        <v>1054</v>
       </c>
       <c r="D58" s="12"/>
       <c r="E58" s="13"/>
     </row>
     <row r="59" ht="13.65" customHeight="1">
       <c r="A59" t="s" s="3">
+        <v>1054</v>
+      </c>
+      <c r="B59" t="s" s="3">
         <v>1055</v>
       </c>
-      <c r="B59" t="s" s="3">
-        <v>1056</v>
-      </c>
       <c r="C59" t="s" s="3">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="D59" s="12"/>
       <c r="E59" s="13"/>
     </row>
     <row r="60" ht="13.65" customHeight="1">
       <c r="A60" t="s" s="3">
+        <v>1056</v>
+      </c>
+      <c r="B60" t="s" s="3">
         <v>1057</v>
       </c>
-      <c r="B60" t="s" s="3">
-        <v>1058</v>
-      </c>
       <c r="C60" t="s" s="3">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="D60" s="12"/>
       <c r="E60" s="13"/>
     </row>
     <row r="61" ht="13.65" customHeight="1">
       <c r="A61" t="s" s="3">
+        <v>1058</v>
+      </c>
+      <c r="B61" t="s" s="3">
         <v>1059</v>
       </c>
-      <c r="B61" t="s" s="3">
-        <v>1060</v>
-      </c>
       <c r="C61" t="s" s="3">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="D61" s="12"/>
       <c r="E61" s="13"/>
     </row>
     <row r="62" ht="13.65" customHeight="1">
       <c r="A62" t="s" s="3">
+        <v>1060</v>
+      </c>
+      <c r="B62" t="s" s="3">
         <v>1061</v>
       </c>
-      <c r="B62" t="s" s="3">
+      <c r="C62" t="s" s="3">
         <v>1062</v>
-      </c>
-      <c r="C62" t="s" s="3">
-        <v>1063</v>
       </c>
       <c r="D62" s="12"/>
       <c r="E62" s="13"/>
     </row>
     <row r="63" ht="13.65" customHeight="1">
       <c r="A63" t="s" s="3">
+        <v>1063</v>
+      </c>
+      <c r="B63" t="s" s="3">
         <v>1064</v>
       </c>
-      <c r="B63" t="s" s="3">
+      <c r="C63" t="s" s="3">
         <v>1065</v>
-      </c>
-      <c r="C63" t="s" s="3">
-        <v>1066</v>
       </c>
       <c r="D63" s="12"/>
       <c r="E63" s="13"/>
     </row>
     <row r="64" ht="13.65" customHeight="1">
       <c r="A64" t="s" s="3">
+        <v>1066</v>
+      </c>
+      <c r="B64" t="s" s="3">
         <v>1067</v>
       </c>
-      <c r="B64" t="s" s="3">
+      <c r="C64" t="s" s="3">
         <v>1068</v>
-      </c>
-      <c r="C64" t="s" s="3">
-        <v>1069</v>
       </c>
       <c r="D64" s="12"/>
       <c r="E64" s="13"/>
     </row>
     <row r="65" ht="13.65" customHeight="1">
       <c r="A65" t="s" s="3">
+        <v>1069</v>
+      </c>
+      <c r="B65" t="s" s="3">
         <v>1070</v>
       </c>
-      <c r="B65" t="s" s="3">
-        <v>1071</v>
-      </c>
       <c r="C65" t="s" s="3">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="D65" s="12"/>
       <c r="E65" s="13"/>
     </row>
     <row r="66" ht="13.65" customHeight="1">
       <c r="A66" t="s" s="3">
+        <v>1071</v>
+      </c>
+      <c r="B66" t="s" s="3">
         <v>1072</v>
       </c>
-      <c r="B66" t="s" s="3">
-        <v>1073</v>
-      </c>
       <c r="C66" t="s" s="3">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="D66" s="12"/>
       <c r="E66" s="13"/>
     </row>
     <row r="67" ht="13.65" customHeight="1">
       <c r="A67" t="s" s="3">
+        <v>1073</v>
+      </c>
+      <c r="B67" t="s" s="3">
         <v>1074</v>
       </c>
-      <c r="B67" t="s" s="3">
-        <v>1075</v>
-      </c>
       <c r="C67" t="s" s="3">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="D67" s="12"/>
       <c r="E67" s="13"/>
     </row>
     <row r="68" ht="13.65" customHeight="1">
       <c r="A68" t="s" s="3">
+        <v>1075</v>
+      </c>
+      <c r="B68" t="s" s="3">
         <v>1076</v>
       </c>
-      <c r="B68" t="s" s="3">
+      <c r="C68" t="s" s="3">
         <v>1077</v>
-      </c>
-      <c r="C68" t="s" s="3">
-        <v>1078</v>
       </c>
       <c r="D68" s="12"/>
       <c r="E68" s="13"/>
     </row>
     <row r="69" ht="13.65" customHeight="1">
       <c r="A69" t="s" s="3">
+        <v>1078</v>
+      </c>
+      <c r="B69" t="s" s="3">
         <v>1079</v>
       </c>
-      <c r="B69" t="s" s="3">
-        <v>1080</v>
-      </c>
       <c r="C69" t="s" s="3">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="D69" s="12"/>
       <c r="E69" s="13"/>
@@ -22117,49 +22114,49 @@
         <v>168</v>
       </c>
       <c r="B70" t="s" s="3">
+        <v>1080</v>
+      </c>
+      <c r="C70" t="s" s="3">
         <v>1081</v>
-      </c>
-      <c r="C70" t="s" s="3">
-        <v>1082</v>
       </c>
       <c r="D70" s="12"/>
       <c r="E70" s="13"/>
     </row>
     <row r="71" ht="13.65" customHeight="1">
       <c r="A71" t="s" s="3">
+        <v>1082</v>
+      </c>
+      <c r="B71" t="s" s="3">
         <v>1083</v>
       </c>
-      <c r="B71" t="s" s="3">
-        <v>1084</v>
-      </c>
       <c r="C71" t="s" s="3">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="D71" s="12"/>
       <c r="E71" s="13"/>
     </row>
     <row r="72" ht="13.65" customHeight="1">
       <c r="A72" t="s" s="3">
+        <v>1084</v>
+      </c>
+      <c r="B72" t="s" s="3">
         <v>1085</v>
       </c>
-      <c r="B72" t="s" s="3">
-        <v>1086</v>
-      </c>
       <c r="C72" t="s" s="3">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D72" s="12"/>
       <c r="E72" s="13"/>
     </row>
     <row r="73" ht="13.65" customHeight="1">
       <c r="A73" t="s" s="3">
+        <v>1086</v>
+      </c>
+      <c r="B73" t="s" s="3">
         <v>1087</v>
       </c>
-      <c r="B73" t="s" s="3">
-        <v>1088</v>
-      </c>
       <c r="C73" t="s" s="3">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="D73" s="12"/>
       <c r="E73" s="13"/>
@@ -22169,49 +22166,49 @@
         <v>195</v>
       </c>
       <c r="B74" t="s" s="3">
+        <v>1088</v>
+      </c>
+      <c r="C74" t="s" s="3">
         <v>1089</v>
-      </c>
-      <c r="C74" t="s" s="3">
-        <v>1090</v>
       </c>
       <c r="D74" s="12"/>
       <c r="E74" s="13"/>
     </row>
     <row r="75" ht="13.65" customHeight="1">
       <c r="A75" t="s" s="3">
+        <v>1090</v>
+      </c>
+      <c r="B75" t="s" s="3">
         <v>1091</v>
       </c>
-      <c r="B75" t="s" s="3">
+      <c r="C75" t="s" s="3">
         <v>1092</v>
-      </c>
-      <c r="C75" t="s" s="3">
-        <v>1093</v>
       </c>
       <c r="D75" s="12"/>
       <c r="E75" s="13"/>
     </row>
     <row r="76" ht="13.65" customHeight="1">
       <c r="A76" t="s" s="3">
+        <v>1093</v>
+      </c>
+      <c r="B76" t="s" s="3">
         <v>1094</v>
       </c>
-      <c r="B76" t="s" s="3">
+      <c r="C76" t="s" s="3">
         <v>1095</v>
-      </c>
-      <c r="C76" t="s" s="3">
-        <v>1096</v>
       </c>
       <c r="D76" s="12"/>
       <c r="E76" s="13"/>
     </row>
     <row r="77" ht="13.65" customHeight="1">
       <c r="A77" t="s" s="3">
+        <v>1096</v>
+      </c>
+      <c r="B77" t="s" s="3">
         <v>1097</v>
       </c>
-      <c r="B77" t="s" s="3">
-        <v>1098</v>
-      </c>
       <c r="C77" t="s" s="3">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="D77" s="12"/>
       <c r="E77" s="13"/>
@@ -22221,543 +22218,543 @@
         <v>238</v>
       </c>
       <c r="B78" t="s" s="3">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="C78" t="s" s="3">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="D78" s="12"/>
       <c r="E78" s="13"/>
     </row>
     <row r="79" ht="13.65" customHeight="1">
       <c r="A79" t="s" s="3">
+        <v>1099</v>
+      </c>
+      <c r="B79" t="s" s="3">
         <v>1100</v>
       </c>
-      <c r="B79" t="s" s="3">
-        <v>1101</v>
-      </c>
       <c r="C79" t="s" s="3">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="D79" s="12"/>
       <c r="E79" s="13"/>
     </row>
     <row r="80" ht="13.65" customHeight="1">
       <c r="A80" t="s" s="3">
+        <v>1101</v>
+      </c>
+      <c r="B80" t="s" s="3">
         <v>1102</v>
       </c>
-      <c r="B80" t="s" s="3">
+      <c r="C80" t="s" s="3">
         <v>1103</v>
-      </c>
-      <c r="C80" t="s" s="3">
-        <v>1104</v>
       </c>
       <c r="D80" s="12"/>
       <c r="E80" s="13"/>
     </row>
     <row r="81" ht="13.65" customHeight="1">
       <c r="A81" t="s" s="3">
+        <v>1104</v>
+      </c>
+      <c r="B81" t="s" s="3">
         <v>1105</v>
       </c>
-      <c r="B81" t="s" s="3">
+      <c r="C81" t="s" s="3">
         <v>1106</v>
-      </c>
-      <c r="C81" t="s" s="3">
-        <v>1107</v>
       </c>
       <c r="D81" s="12"/>
       <c r="E81" s="13"/>
     </row>
     <row r="82" ht="13.65" customHeight="1">
       <c r="A82" t="s" s="3">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="B82" t="s" s="3">
+        <v>941</v>
+      </c>
+      <c r="C82" t="s" s="3">
         <v>942</v>
-      </c>
-      <c r="C82" t="s" s="3">
-        <v>943</v>
       </c>
       <c r="D82" s="12"/>
       <c r="E82" s="13"/>
     </row>
     <row r="83" ht="13.65" customHeight="1">
       <c r="A83" t="s" s="3">
+        <v>1108</v>
+      </c>
+      <c r="B83" t="s" s="3">
         <v>1109</v>
       </c>
-      <c r="B83" t="s" s="3">
+      <c r="C83" t="s" s="3">
         <v>1110</v>
-      </c>
-      <c r="C83" t="s" s="3">
-        <v>1111</v>
       </c>
       <c r="D83" s="12"/>
       <c r="E83" s="13"/>
     </row>
     <row r="84" ht="13.65" customHeight="1">
       <c r="A84" t="s" s="6">
+        <v>1111</v>
+      </c>
+      <c r="B84" t="s" s="6">
         <v>1112</v>
       </c>
-      <c r="B84" t="s" s="6">
+      <c r="C84" t="s" s="6">
         <v>1113</v>
-      </c>
-      <c r="C84" t="s" s="6">
-        <v>1114</v>
       </c>
       <c r="D84" s="12"/>
       <c r="E84" s="13"/>
     </row>
     <row r="85" ht="13.65" customHeight="1">
       <c r="A85" t="s" s="6">
+        <v>1114</v>
+      </c>
+      <c r="B85" t="s" s="6">
         <v>1115</v>
       </c>
-      <c r="B85" t="s" s="6">
+      <c r="C85" t="s" s="6">
         <v>1116</v>
-      </c>
-      <c r="C85" t="s" s="6">
-        <v>1117</v>
       </c>
       <c r="D85" s="12"/>
       <c r="E85" s="13"/>
     </row>
     <row r="86" ht="13.65" customHeight="1">
       <c r="A86" t="s" s="6">
+        <v>1117</v>
+      </c>
+      <c r="B86" t="s" s="6">
         <v>1118</v>
       </c>
-      <c r="B86" t="s" s="6">
+      <c r="C86" t="s" s="6">
         <v>1119</v>
-      </c>
-      <c r="C86" t="s" s="6">
-        <v>1120</v>
       </c>
       <c r="D86" s="12"/>
       <c r="E86" s="13"/>
     </row>
     <row r="87" ht="13.65" customHeight="1">
       <c r="A87" t="s" s="6">
+        <v>1120</v>
+      </c>
+      <c r="B87" t="s" s="6">
         <v>1121</v>
       </c>
-      <c r="B87" t="s" s="6">
+      <c r="C87" t="s" s="6">
         <v>1122</v>
-      </c>
-      <c r="C87" t="s" s="6">
-        <v>1123</v>
       </c>
       <c r="D87" s="12"/>
       <c r="E87" s="13"/>
     </row>
     <row r="88" ht="13.65" customHeight="1">
       <c r="A88" t="s" s="6">
+        <v>1123</v>
+      </c>
+      <c r="B88" t="s" s="6">
         <v>1124</v>
       </c>
-      <c r="B88" t="s" s="6">
+      <c r="C88" t="s" s="6">
         <v>1125</v>
-      </c>
-      <c r="C88" t="s" s="6">
-        <v>1126</v>
       </c>
       <c r="D88" s="12"/>
       <c r="E88" s="13"/>
     </row>
     <row r="89" ht="13.65" customHeight="1">
       <c r="A89" t="s" s="6">
+        <v>1126</v>
+      </c>
+      <c r="B89" t="s" s="6">
         <v>1127</v>
       </c>
-      <c r="B89" t="s" s="6">
+      <c r="C89" t="s" s="6">
         <v>1128</v>
-      </c>
-      <c r="C89" t="s" s="6">
-        <v>1129</v>
       </c>
       <c r="D89" s="12"/>
       <c r="E89" s="13"/>
     </row>
     <row r="90" ht="13.65" customHeight="1">
       <c r="A90" t="s" s="6">
+        <v>1129</v>
+      </c>
+      <c r="B90" t="s" s="6">
         <v>1130</v>
       </c>
-      <c r="B90" t="s" s="6">
+      <c r="C90" t="s" s="6">
         <v>1131</v>
-      </c>
-      <c r="C90" t="s" s="6">
-        <v>1132</v>
       </c>
       <c r="D90" s="12"/>
       <c r="E90" s="13"/>
     </row>
     <row r="91" ht="13.65" customHeight="1">
       <c r="A91" t="s" s="6">
+        <v>1132</v>
+      </c>
+      <c r="B91" t="s" s="6">
         <v>1133</v>
       </c>
-      <c r="B91" t="s" s="6">
+      <c r="C91" t="s" s="6">
         <v>1134</v>
-      </c>
-      <c r="C91" t="s" s="6">
-        <v>1135</v>
       </c>
       <c r="D91" s="12"/>
       <c r="E91" s="13"/>
     </row>
     <row r="92" ht="13.65" customHeight="1">
       <c r="A92" t="s" s="6">
+        <v>1135</v>
+      </c>
+      <c r="B92" t="s" s="6">
         <v>1136</v>
       </c>
-      <c r="B92" t="s" s="6">
+      <c r="C92" t="s" s="6">
         <v>1137</v>
-      </c>
-      <c r="C92" t="s" s="6">
-        <v>1138</v>
       </c>
       <c r="D92" s="12"/>
       <c r="E92" s="13"/>
     </row>
     <row r="93" ht="13.65" customHeight="1">
       <c r="A93" t="s" s="6">
+        <v>1138</v>
+      </c>
+      <c r="B93" t="s" s="6">
         <v>1139</v>
       </c>
-      <c r="B93" t="s" s="6">
-        <v>1140</v>
-      </c>
       <c r="C93" t="s" s="6">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="D93" s="12"/>
       <c r="E93" s="13"/>
     </row>
     <row r="94" ht="13.65" customHeight="1">
       <c r="A94" t="s" s="6">
+        <v>1140</v>
+      </c>
+      <c r="B94" t="s" s="6">
         <v>1141</v>
       </c>
-      <c r="B94" t="s" s="6">
+      <c r="C94" t="s" s="6">
         <v>1142</v>
-      </c>
-      <c r="C94" t="s" s="6">
-        <v>1143</v>
       </c>
       <c r="D94" s="12"/>
       <c r="E94" s="13"/>
     </row>
     <row r="95" ht="13.65" customHeight="1">
       <c r="A95" t="s" s="6">
+        <v>1143</v>
+      </c>
+      <c r="B95" t="s" s="6">
         <v>1144</v>
       </c>
-      <c r="B95" t="s" s="6">
-        <v>1145</v>
-      </c>
       <c r="C95" t="s" s="6">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="D95" s="12"/>
       <c r="E95" s="13"/>
     </row>
     <row r="96" ht="13.65" customHeight="1">
       <c r="A96" t="s" s="6">
+        <v>1145</v>
+      </c>
+      <c r="B96" t="s" s="6">
         <v>1146</v>
       </c>
-      <c r="B96" t="s" s="6">
+      <c r="C96" t="s" s="6">
         <v>1147</v>
-      </c>
-      <c r="C96" t="s" s="6">
-        <v>1148</v>
       </c>
       <c r="D96" s="12"/>
       <c r="E96" s="13"/>
     </row>
     <row r="97" ht="13.65" customHeight="1">
       <c r="A97" t="s" s="6">
+        <v>1148</v>
+      </c>
+      <c r="B97" t="s" s="6">
         <v>1149</v>
       </c>
-      <c r="B97" t="s" s="6">
+      <c r="C97" t="s" s="6">
         <v>1150</v>
-      </c>
-      <c r="C97" t="s" s="6">
-        <v>1151</v>
       </c>
       <c r="D97" s="12"/>
       <c r="E97" s="13"/>
     </row>
     <row r="98" ht="13.65" customHeight="1">
       <c r="A98" t="s" s="6">
+        <v>1151</v>
+      </c>
+      <c r="B98" t="s" s="6">
         <v>1152</v>
       </c>
-      <c r="B98" t="s" s="6">
+      <c r="C98" t="s" s="6">
         <v>1153</v>
-      </c>
-      <c r="C98" t="s" s="6">
-        <v>1154</v>
       </c>
       <c r="D98" s="12"/>
       <c r="E98" s="13"/>
     </row>
     <row r="99" ht="13.65" customHeight="1">
       <c r="A99" t="s" s="6">
+        <v>1154</v>
+      </c>
+      <c r="B99" t="s" s="6">
         <v>1155</v>
       </c>
-      <c r="B99" t="s" s="6">
-        <v>1156</v>
-      </c>
       <c r="C99" t="s" s="6">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="D99" s="12"/>
       <c r="E99" s="13"/>
     </row>
     <row r="100" ht="13.65" customHeight="1">
       <c r="A100" t="s" s="6">
+        <v>1156</v>
+      </c>
+      <c r="B100" t="s" s="6">
         <v>1157</v>
       </c>
-      <c r="B100" t="s" s="6">
+      <c r="C100" t="s" s="6">
         <v>1158</v>
-      </c>
-      <c r="C100" t="s" s="6">
-        <v>1159</v>
       </c>
       <c r="D100" s="12"/>
       <c r="E100" s="13"/>
     </row>
     <row r="101" ht="13.65" customHeight="1">
       <c r="A101" t="s" s="6">
+        <v>1159</v>
+      </c>
+      <c r="B101" t="s" s="6">
         <v>1160</v>
       </c>
-      <c r="B101" t="s" s="6">
+      <c r="C101" t="s" s="6">
         <v>1161</v>
-      </c>
-      <c r="C101" t="s" s="6">
-        <v>1162</v>
       </c>
       <c r="D101" s="12"/>
       <c r="E101" s="13"/>
     </row>
     <row r="102" ht="13.65" customHeight="1">
       <c r="A102" t="s" s="6">
+        <v>1162</v>
+      </c>
+      <c r="B102" t="s" s="6">
         <v>1163</v>
       </c>
-      <c r="B102" t="s" s="6">
+      <c r="C102" t="s" s="6">
         <v>1164</v>
-      </c>
-      <c r="C102" t="s" s="6">
-        <v>1165</v>
       </c>
       <c r="D102" s="12"/>
       <c r="E102" s="13"/>
     </row>
     <row r="103" ht="13.65" customHeight="1">
       <c r="A103" t="s" s="6">
+        <v>1165</v>
+      </c>
+      <c r="B103" t="s" s="6">
         <v>1166</v>
       </c>
-      <c r="B103" t="s" s="6">
+      <c r="C103" t="s" s="6">
         <v>1167</v>
-      </c>
-      <c r="C103" t="s" s="6">
-        <v>1168</v>
       </c>
       <c r="D103" s="12"/>
       <c r="E103" s="13"/>
     </row>
     <row r="104" ht="13.65" customHeight="1">
       <c r="A104" t="s" s="6">
+        <v>1168</v>
+      </c>
+      <c r="B104" t="s" s="6">
         <v>1169</v>
       </c>
-      <c r="B104" t="s" s="6">
+      <c r="C104" t="s" s="6">
         <v>1170</v>
-      </c>
-      <c r="C104" t="s" s="6">
-        <v>1171</v>
       </c>
       <c r="D104" s="12"/>
       <c r="E104" s="13"/>
     </row>
     <row r="105" ht="13.65" customHeight="1">
       <c r="A105" t="s" s="6">
+        <v>1171</v>
+      </c>
+      <c r="B105" t="s" s="6">
         <v>1172</v>
       </c>
-      <c r="B105" t="s" s="6">
-        <v>1173</v>
-      </c>
       <c r="C105" t="s" s="6">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="D105" s="12"/>
       <c r="E105" s="13"/>
     </row>
     <row r="106" ht="13.65" customHeight="1">
       <c r="A106" t="s" s="6">
+        <v>1173</v>
+      </c>
+      <c r="B106" t="s" s="6">
         <v>1174</v>
       </c>
-      <c r="B106" t="s" s="6">
+      <c r="C106" t="s" s="6">
         <v>1175</v>
-      </c>
-      <c r="C106" t="s" s="6">
-        <v>1176</v>
       </c>
       <c r="D106" s="12"/>
       <c r="E106" s="13"/>
     </row>
     <row r="107" ht="13.65" customHeight="1">
       <c r="A107" t="s" s="6">
+        <v>1176</v>
+      </c>
+      <c r="B107" t="s" s="6">
         <v>1177</v>
       </c>
-      <c r="B107" t="s" s="6">
+      <c r="C107" t="s" s="6">
         <v>1178</v>
-      </c>
-      <c r="C107" t="s" s="6">
-        <v>1179</v>
       </c>
       <c r="D107" s="12"/>
       <c r="E107" s="13"/>
     </row>
     <row r="108" ht="13.65" customHeight="1">
       <c r="A108" t="s" s="6">
+        <v>1179</v>
+      </c>
+      <c r="B108" t="s" s="6">
         <v>1180</v>
       </c>
-      <c r="B108" t="s" s="6">
-        <v>1181</v>
-      </c>
       <c r="C108" t="s" s="6">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="D108" s="12"/>
       <c r="E108" s="13"/>
     </row>
     <row r="109" ht="13.65" customHeight="1">
       <c r="A109" t="s" s="6">
+        <v>1181</v>
+      </c>
+      <c r="B109" t="s" s="6">
         <v>1182</v>
       </c>
-      <c r="B109" t="s" s="6">
-        <v>1183</v>
-      </c>
       <c r="C109" t="s" s="6">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="D109" s="12"/>
       <c r="E109" s="13"/>
     </row>
     <row r="110" ht="13.65" customHeight="1">
       <c r="A110" t="s" s="6">
+        <v>1183</v>
+      </c>
+      <c r="B110" t="s" s="6">
         <v>1184</v>
       </c>
-      <c r="B110" t="s" s="6">
-        <v>1185</v>
-      </c>
       <c r="C110" t="s" s="6">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="D110" s="12"/>
       <c r="E110" s="13"/>
     </row>
     <row r="111" ht="13.65" customHeight="1">
       <c r="A111" t="s" s="6">
+        <v>1185</v>
+      </c>
+      <c r="B111" t="s" s="6">
         <v>1186</v>
       </c>
-      <c r="B111" t="s" s="6">
+      <c r="C111" t="s" s="6">
         <v>1187</v>
-      </c>
-      <c r="C111" t="s" s="6">
-        <v>1188</v>
       </c>
       <c r="D111" s="12"/>
       <c r="E111" s="13"/>
     </row>
     <row r="112" ht="13.65" customHeight="1">
       <c r="A112" t="s" s="6">
+        <v>1188</v>
+      </c>
+      <c r="B112" t="s" s="6">
         <v>1189</v>
       </c>
-      <c r="B112" t="s" s="6">
-        <v>1190</v>
-      </c>
       <c r="C112" t="s" s="6">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="D112" s="12"/>
       <c r="E112" s="13"/>
     </row>
     <row r="113" ht="13.65" customHeight="1">
       <c r="A113" t="s" s="6">
+        <v>1190</v>
+      </c>
+      <c r="B113" t="s" s="6">
         <v>1191</v>
       </c>
-      <c r="B113" t="s" s="6">
+      <c r="C113" t="s" s="6">
         <v>1192</v>
-      </c>
-      <c r="C113" t="s" s="6">
-        <v>1193</v>
       </c>
       <c r="D113" s="12"/>
       <c r="E113" s="13"/>
     </row>
     <row r="114" ht="13.65" customHeight="1">
       <c r="A114" t="s" s="6">
+        <v>1193</v>
+      </c>
+      <c r="B114" t="s" s="6">
         <v>1194</v>
       </c>
-      <c r="B114" t="s" s="6">
-        <v>1195</v>
-      </c>
       <c r="C114" t="s" s="6">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="D114" s="12"/>
       <c r="E114" s="13"/>
     </row>
     <row r="115" ht="13.65" customHeight="1">
       <c r="A115" t="s" s="6">
+        <v>1195</v>
+      </c>
+      <c r="B115" t="s" s="6">
         <v>1196</v>
       </c>
-      <c r="B115" t="s" s="6">
-        <v>1197</v>
-      </c>
       <c r="C115" t="s" s="6">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D115" s="12"/>
       <c r="E115" s="13"/>
     </row>
     <row r="116" ht="13.65" customHeight="1">
       <c r="A116" t="s" s="6">
+        <v>1197</v>
+      </c>
+      <c r="B116" t="s" s="6">
         <v>1198</v>
       </c>
-      <c r="B116" t="s" s="6">
-        <v>1199</v>
-      </c>
       <c r="C116" t="s" s="6">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="D116" s="12"/>
       <c r="E116" s="13"/>
     </row>
     <row r="117" ht="13.65" customHeight="1">
       <c r="A117" t="s" s="6">
+        <v>1199</v>
+      </c>
+      <c r="B117" t="s" s="6">
         <v>1200</v>
       </c>
-      <c r="B117" t="s" s="6">
+      <c r="C117" t="s" s="6">
         <v>1201</v>
-      </c>
-      <c r="C117" t="s" s="6">
-        <v>1202</v>
       </c>
       <c r="D117" s="12"/>
       <c r="E117" s="13"/>
     </row>
     <row r="118" ht="13.65" customHeight="1">
       <c r="A118" t="s" s="6">
+        <v>1202</v>
+      </c>
+      <c r="B118" t="s" s="6">
         <v>1203</v>
       </c>
-      <c r="B118" t="s" s="6">
-        <v>1204</v>
-      </c>
       <c r="C118" t="s" s="6">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="D118" s="12"/>
       <c r="E118" s="13"/>
     </row>
     <row r="119" ht="13.65" customHeight="1">
       <c r="A119" t="s" s="6">
+        <v>1204</v>
+      </c>
+      <c r="B119" t="s" s="6">
         <v>1205</v>
       </c>
-      <c r="B119" t="s" s="6">
-        <v>1206</v>
-      </c>
       <c r="C119" t="s" s="6">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="D119" s="12"/>
       <c r="E119" s="13"/>
@@ -22767,192 +22764,192 @@
         <v>205</v>
       </c>
       <c r="B120" t="s" s="6">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="C120" t="s" s="6">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="D120" s="12"/>
       <c r="E120" s="13"/>
     </row>
     <row r="121" ht="13.65" customHeight="1">
       <c r="A121" t="s" s="6">
+        <v>1206</v>
+      </c>
+      <c r="B121" t="s" s="6">
         <v>1207</v>
       </c>
-      <c r="B121" t="s" s="6">
+      <c r="C121" t="s" s="6">
         <v>1208</v>
-      </c>
-      <c r="C121" t="s" s="6">
-        <v>1209</v>
       </c>
       <c r="D121" s="12"/>
       <c r="E121" s="13"/>
     </row>
     <row r="122" ht="13.65" customHeight="1">
       <c r="A122" t="s" s="6">
+        <v>1209</v>
+      </c>
+      <c r="B122" t="s" s="6">
         <v>1210</v>
       </c>
-      <c r="B122" t="s" s="6">
+      <c r="C122" t="s" s="6">
         <v>1211</v>
-      </c>
-      <c r="C122" t="s" s="6">
-        <v>1212</v>
       </c>
       <c r="D122" s="12"/>
       <c r="E122" s="13"/>
     </row>
     <row r="123" ht="13.65" customHeight="1">
       <c r="A123" t="s" s="6">
+        <v>1212</v>
+      </c>
+      <c r="B123" t="s" s="6">
         <v>1213</v>
       </c>
-      <c r="B123" t="s" s="6">
+      <c r="C123" t="s" s="6">
         <v>1214</v>
-      </c>
-      <c r="C123" t="s" s="6">
-        <v>1215</v>
       </c>
       <c r="D123" s="12"/>
       <c r="E123" s="13"/>
     </row>
     <row r="124" ht="13.65" customHeight="1">
       <c r="A124" t="s" s="6">
+        <v>1215</v>
+      </c>
+      <c r="B124" t="s" s="6">
         <v>1216</v>
       </c>
-      <c r="B124" t="s" s="6">
+      <c r="C124" t="s" s="6">
         <v>1217</v>
-      </c>
-      <c r="C124" t="s" s="6">
-        <v>1218</v>
       </c>
       <c r="D124" s="12"/>
       <c r="E124" s="13"/>
     </row>
     <row r="125" ht="13.65" customHeight="1">
       <c r="A125" t="s" s="6">
+        <v>1218</v>
+      </c>
+      <c r="B125" t="s" s="6">
         <v>1219</v>
       </c>
-      <c r="B125" t="s" s="6">
+      <c r="C125" t="s" s="6">
         <v>1220</v>
-      </c>
-      <c r="C125" t="s" s="6">
-        <v>1221</v>
       </c>
       <c r="D125" s="12"/>
       <c r="E125" s="13"/>
     </row>
     <row r="126" ht="13.65" customHeight="1">
       <c r="A126" t="s" s="6">
+        <v>1221</v>
+      </c>
+      <c r="B126" t="s" s="6">
         <v>1222</v>
       </c>
-      <c r="B126" t="s" s="6">
+      <c r="C126" t="s" s="6">
         <v>1223</v>
-      </c>
-      <c r="C126" t="s" s="6">
-        <v>1224</v>
       </c>
       <c r="D126" s="12"/>
       <c r="E126" s="13"/>
     </row>
     <row r="127" ht="13.65" customHeight="1">
       <c r="A127" t="s" s="6">
+        <v>1224</v>
+      </c>
+      <c r="B127" t="s" s="14">
         <v>1225</v>
       </c>
-      <c r="B127" t="s" s="14">
+      <c r="C127" t="s" s="6">
         <v>1226</v>
-      </c>
-      <c r="C127" t="s" s="6">
-        <v>1227</v>
       </c>
       <c r="D127" s="12"/>
       <c r="E127" s="13"/>
     </row>
     <row r="128" ht="13.65" customHeight="1">
       <c r="A128" t="s" s="6">
+        <v>1227</v>
+      </c>
+      <c r="B128" t="s" s="6">
         <v>1228</v>
       </c>
-      <c r="B128" t="s" s="6">
-        <v>1229</v>
-      </c>
       <c r="C128" t="s" s="6">
-        <v>1229</v>
+        <v>1228</v>
       </c>
       <c r="D128" s="12"/>
       <c r="E128" s="13"/>
     </row>
     <row r="129" ht="13.65" customHeight="1">
       <c r="A129" t="s" s="6">
+        <v>1229</v>
+      </c>
+      <c r="B129" t="s" s="6">
         <v>1230</v>
       </c>
-      <c r="B129" t="s" s="6">
+      <c r="C129" t="s" s="6">
         <v>1231</v>
-      </c>
-      <c r="C129" t="s" s="6">
-        <v>1232</v>
       </c>
       <c r="D129" s="12"/>
       <c r="E129" s="13"/>
     </row>
     <row r="130" ht="13.65" customHeight="1">
       <c r="A130" t="s" s="6">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B130" t="s" s="6">
-        <v>1233</v>
+        <v>1232</v>
       </c>
       <c r="C130" t="s" s="6">
-        <v>1233</v>
+        <v>1232</v>
       </c>
       <c r="D130" s="12"/>
       <c r="E130" s="13"/>
     </row>
     <row r="131" ht="13.65" customHeight="1">
       <c r="A131" t="s" s="6">
+        <v>1233</v>
+      </c>
+      <c r="B131" t="s" s="6">
         <v>1234</v>
       </c>
-      <c r="B131" t="s" s="6">
-        <v>1235</v>
-      </c>
       <c r="C131" t="s" s="6">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="D131" s="12"/>
       <c r="E131" s="13"/>
     </row>
     <row r="132" ht="13.65" customHeight="1">
       <c r="A132" t="s" s="6">
+        <v>1235</v>
+      </c>
+      <c r="B132" t="s" s="6">
         <v>1236</v>
       </c>
-      <c r="B132" t="s" s="6">
-        <v>1237</v>
-      </c>
       <c r="C132" t="s" s="6">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="D132" s="12"/>
       <c r="E132" s="13"/>
     </row>
     <row r="133" ht="13.65" customHeight="1">
       <c r="A133" t="s" s="6">
+        <v>1237</v>
+      </c>
+      <c r="B133" t="s" s="6">
         <v>1238</v>
       </c>
-      <c r="B133" t="s" s="6">
+      <c r="C133" t="s" s="6">
         <v>1239</v>
-      </c>
-      <c r="C133" t="s" s="6">
-        <v>1240</v>
       </c>
       <c r="D133" s="12"/>
       <c r="E133" s="13"/>
     </row>
     <row r="134" ht="13.65" customHeight="1">
       <c r="A134" t="s" s="6">
+        <v>1240</v>
+      </c>
+      <c r="B134" t="s" s="6">
         <v>1241</v>
       </c>
-      <c r="B134" t="s" s="6">
+      <c r="C134" t="s" s="6">
         <v>1242</v>
-      </c>
-      <c r="C134" t="s" s="6">
-        <v>1243</v>
       </c>
       <c r="D134" s="15"/>
       <c r="E134" s="16"/>

</xml_diff>